<commit_message>
Remove legacy site and update thesis documentation
Deleted the _site directory and related HTML, PDF, and asset files to remove the legacy Quarto site build. Updated and reorganized documentation in the docs directory, including renaming about.html to summary.html, updating Excel and PDF files, and adding a new image. This streamlines the project structure and focuses on the current documentation.
</commit_message>
<xml_diff>
--- a/docs/Codebook_Cigarette.xlsx
+++ b/docs/Codebook_Cigarette.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\myechow\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Graduate Courses\PHPH 7990\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D289B9F6-6AD4-44AD-9D74-66870981D8F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB777CB4-6A11-4981-8838-C3B6D7A4A91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22780" windowHeight="14540" xr2:uid="{576F2D76-5E76-4B83-A195-30915DF4AE14}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="67">
   <si>
     <t>att1</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>How many of your friends would you estimate smoke cigarettes?</t>
-  </si>
-  <si>
-    <t>1="All" 2="Most" 3="Some" 4="A Few" 5="None"</t>
   </si>
   <si>
     <t>des2</t>
@@ -110,10 +107,10 @@
     <t>Which grade are you in?</t>
   </si>
   <si>
-    <t>V7666</t>
+    <t>plh1</t>
   </si>
   <si>
-    <t>1="Definitely yes" 2="Probably yes" 3="Probably not" 4="Definitely not"</t>
+    <t>V7666</t>
   </si>
   <si>
     <t>Have you smoked cigarettes in the past 30 days?</t>
@@ -215,9 +212,6 @@
     <t>V7206,V7207</t>
   </si>
   <si>
-    <t>Would you consider trying tobacco if one of your closest friends offered it to you?</t>
-  </si>
-  <si>
     <t>0= Eghth, 1= Tenth</t>
   </si>
   <si>
@@ -231,6 +225,18 @@
   </si>
   <si>
     <t>How do you think your close friends would feel about you smoking cigarettes occasionally?</t>
+  </si>
+  <si>
+    <t>If one of your closest friends offered you a cigarette, how confident are you that you could refuse it?</t>
+  </si>
+  <si>
+    <t>1 = "Not at all confident" 2 =" Slightly confident" "3 = Moderately confident" 4 = "Very confident"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">*Sample Weights were applied </t>
+  </si>
+  <si>
+    <t>1="None" 2="A Few" 3="Some" 4="Most" 5="All"</t>
   </si>
 </sst>
 </file>
@@ -536,7 +542,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -664,29 +670,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1035,16 +1018,16 @@
   <sheetData>
     <row r="1" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="46" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="47"/>
+      <c r="A2" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="38"/>
       <c r="C2" s="37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D2" s="38"/>
       <c r="E2" s="23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1058,7 +1041,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>1</v>
@@ -1069,55 +1052,55 @@
         <v>3</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" s="16" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E4" s="29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="22" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E5" s="30" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="45"/>
+      <c r="A6" s="33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="39"/>
       <c r="C6" s="39" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D6" s="39"/>
       <c r="E6" s="32"/>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>7</v>
@@ -1128,28 +1111,28 @@
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="29" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="44" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="45"/>
+      <c r="A9" s="33" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="39"/>
       <c r="C9" s="39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D9" s="39"/>
       <c r="E9" s="32"/>
@@ -1165,7 +1148,7 @@
         <v>8</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>9</v>
@@ -1173,210 +1156,210 @@
     </row>
     <row r="11" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>11</v>
+        <v>66</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="44" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="48"/>
+      <c r="A12" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="34"/>
       <c r="C12" s="33" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D12" s="34"/>
       <c r="E12" s="14"/>
     </row>
     <row r="13" spans="1:5" s="2" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="E13" s="29" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="44" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" s="48"/>
+      <c r="A14" s="33" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="34"/>
       <c r="C14" s="33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D14" s="34"/>
       <c r="E14" s="10"/>
     </row>
     <row r="15" spans="1:5" s="2" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="29" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" s="2" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="B15" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="16" t="s">
+      <c r="B16" s="41"/>
+      <c r="C16" s="40" t="s">
         <v>36</v>
-      </c>
-      <c r="D15" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="29" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" s="2" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="49" t="s">
-        <v>37</v>
-      </c>
-      <c r="B16" s="50"/>
-      <c r="C16" s="40" t="s">
-        <v>37</v>
       </c>
       <c r="D16" s="41"/>
       <c r="E16" s="10"/>
     </row>
     <row r="17" spans="1:5" s="2" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="31" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C17" s="28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E17" s="29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="1:5" s="2" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="44" t="s">
-        <v>41</v>
-      </c>
-      <c r="B18" s="48"/>
+      <c r="A18" s="33" t="s">
+        <v>40</v>
+      </c>
+      <c r="B18" s="34"/>
       <c r="C18" s="42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D18" s="43"/>
       <c r="E18" s="14"/>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="51" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="52"/>
+      <c r="A20" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="36"/>
       <c r="C20" s="35" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D20" s="36"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>54</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="B21" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>15</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D22" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="B23" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="E24" s="8" t="s">
         <v>21</v>
-      </c>
-      <c r="B24" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="E24" s="8" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1387,7 +1370,9 @@
       <c r="E25" s="21"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="21"/>
+      <c r="A26" s="21" t="s">
+        <v>65</v>
+      </c>
       <c r="B26" s="21"/>
       <c r="C26" s="21"/>
       <c r="D26" s="21"/>
@@ -6890,7 +6875,9 @@
       <c r="E813" s="12"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="16">
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A20:B20"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C9:D9"/>
@@ -6899,6 +6886,12 @@
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C18:D18"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A16:B16"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>